<commit_message>
Tighten verification and accessibility
</commit_message>
<xml_diff>
--- a/public/downloads/retribuciones_mir_2026.xlsx
+++ b/public/downloads/retribuciones_mir_2026.xlsx
@@ -915,7 +915,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>SIMEG + SIMPA</t>
+          <t>SIMEG</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>SIMEG + ICS</t>
+          <t>SIMEG</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>SIMEG + SM Navarra</t>
+          <t>SIMEG</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">

</xml_diff>

<commit_message>
Use 35h annualized MIR hourly model
</commit_message>
<xml_diff>
--- a/public/downloads/retribuciones_mir_2026.xlsx
+++ b/public/downloads/retribuciones_mir_2026.xlsx
@@ -20,8 +20,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
+  </numFmts>
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,6 +35,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font/>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -69,7 +76,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -84,6 +91,22 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2044,10 +2067,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
@@ -2056,234 +2079,362 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Métrica</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>R3</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>R4</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>R5</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>Bruto medio sin guardias €/mes</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="7" t="n">
         <v>1447</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="7" t="n">
         <v>1555</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="7" t="n">
         <v>1694</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="7" t="n">
         <v>1833</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="7" t="n">
         <v>1973</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Bruto medio cartel/80h €/mes</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="7" t="n">
         <v>2806</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="7" t="n">
         <v>3114</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="7" t="n">
         <v>3452</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="7" t="n">
         <v>3790</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="7" t="n">
         <v>3929</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Neto medio cartel/80h €/mes</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="7" t="n">
         <v>2087</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="7" t="n">
         <v>2284</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="7" t="n">
         <v>2486</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="7" t="n">
         <v>2684</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="7" t="n">
         <v>2758</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Guardias como % del bruto total</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="8" t="n">
         <v>0.484</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="8" t="n">
         <v>0.501</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="8" t="n">
         <v>0.509</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="8" t="n">
         <v>0.516</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="8" t="n">
         <v>0.498</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Horas ordinarias/mes usadas</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>162.5</v>
-      </c>
-      <c r="C6" t="n">
-        <v>162.5</v>
-      </c>
-      <c r="D6" t="n">
-        <v>162.5</v>
-      </c>
-      <c r="E6" t="n">
-        <v>162.5</v>
-      </c>
-      <c r="F6" t="n">
-        <v>162.5</v>
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Horas ordinarias/mes usadas (35h semanal anualizada)</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>151.6666666666667</v>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>151.6666666666667</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>151.6666666666667</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>151.6666666666667</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>151.6666666666667</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Horas de guardia/mes usadas</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="7" t="n">
         <v>80</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" s="7" t="n">
         <v>80</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="7" t="n">
         <v>80</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="7" t="n">
         <v>80</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="7" t="n">
         <v>80</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>Horas totales/mes</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>242.5</v>
-      </c>
-      <c r="C8" t="n">
-        <v>242.5</v>
-      </c>
-      <c r="D8" t="n">
-        <v>242.5</v>
-      </c>
-      <c r="E8" t="n">
-        <v>242.5</v>
-      </c>
-      <c r="F8" t="n">
-        <v>242.5</v>
+      <c r="B8" s="9" t="n">
+        <v>231.6666666666667</v>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>231.6666666666667</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>231.6666666666667</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>231.6666666666667</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>231.6666666666667</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Neto €/h real con 80h</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>8.609999999999999</v>
-      </c>
-      <c r="C9" t="n">
-        <v>9.42</v>
-      </c>
-      <c r="D9" t="n">
-        <v>10.25</v>
-      </c>
-      <c r="E9" t="n">
-        <v>11.07</v>
-      </c>
-      <c r="F9" t="n">
-        <v>11.37</v>
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Neto €/h real con 80h (35h/sem anualizadas)</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="n">
+        <v>9.00863309352518</v>
+      </c>
+      <c r="C9" s="10" t="n">
+        <v>9.858992805755395</v>
+      </c>
+      <c r="D9" s="10" t="n">
+        <v>10.73093525179856</v>
+      </c>
+      <c r="E9" s="10" t="n">
+        <v>11.58561151079137</v>
+      </c>
+      <c r="F9" s="10" t="n">
+        <v>11.90503597122302</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Neto €/h con 80h + 5h/sem formacion</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>7.9</v>
-      </c>
-      <c r="C10" t="n">
-        <v>8.65</v>
-      </c>
-      <c r="D10" t="n">
-        <v>9.41</v>
-      </c>
-      <c r="E10" t="n">
-        <v>10.16</v>
-      </c>
-      <c r="F10" t="n">
-        <v>10.44</v>
-      </c>
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Neto €/h si aplica 37,5h/semana</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="n">
+        <v>8.606185567010309</v>
+      </c>
+      <c r="C10" s="10" t="n">
+        <v>9.418556701030928</v>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>10.25154639175258</v>
+      </c>
+      <c r="E10" s="10" t="n">
+        <v>11.0680412371134</v>
+      </c>
+      <c r="F10" s="10" t="n">
+        <v>11.37319587628866</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Nota metodológica</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>35h x 52 / 12 = 151,7h/mes; 151,7 + 80 = 231,7h/mes</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="n"/>
+      <c r="D11" s="7" t="n"/>
+      <c r="E11" s="7" t="n"/>
+      <c r="F11" s="7" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="n"/>
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
+      <c r="F12" s="11" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="n"/>
+      <c r="B13" s="11" t="n"/>
+      <c r="C13" s="11" t="n"/>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="11" t="n"/>
+      <c r="F13" s="11" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="11" t="n"/>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
+      <c r="F14" s="11" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="n"/>
+      <c r="B15" s="11" t="n"/>
+      <c r="C15" s="11" t="n"/>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="11" t="n"/>
+      <c r="F15" s="11" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="11" t="n"/>
+      <c r="F16" s="11" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="n"/>
+      <c r="B17" s="11" t="n"/>
+      <c r="C17" s="11" t="n"/>
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="11" t="n"/>
+      <c r="F17" s="11" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="n"/>
+      <c r="B18" s="11" t="n"/>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="n"/>
+      <c r="F18" s="11" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="n"/>
+      <c r="B19" s="11" t="n"/>
+      <c r="C19" s="11" t="n"/>
+      <c r="D19" s="11" t="n"/>
+      <c r="E19" s="11" t="n"/>
+      <c r="F19" s="11" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="n"/>
+      <c r="B20" s="11" t="n"/>
+      <c r="C20" s="11" t="n"/>
+      <c r="D20" s="11" t="n"/>
+      <c r="E20" s="11" t="n"/>
+      <c r="F20" s="11" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="n"/>
+      <c r="B21" s="11" t="n"/>
+      <c r="C21" s="11" t="n"/>
+      <c r="D21" s="11" t="n"/>
+      <c r="E21" s="11" t="n"/>
+      <c r="F21" s="11" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="n"/>
+      <c r="B22" s="11" t="n"/>
+      <c r="C22" s="11" t="n"/>
+      <c r="D22" s="11" t="n"/>
+      <c r="E22" s="11" t="n"/>
+      <c r="F22" s="11" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="n"/>
+      <c r="B23" s="11" t="n"/>
+      <c r="C23" s="11" t="n"/>
+      <c r="D23" s="11" t="n"/>
+      <c r="E23" s="11" t="n"/>
+      <c r="F23" s="11" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="n"/>
+      <c r="B24" s="11" t="n"/>
+      <c r="C24" s="11" t="n"/>
+      <c r="D24" s="11" t="n"/>
+      <c r="E24" s="11" t="n"/>
+      <c r="F24" s="11" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="n"/>
+      <c r="B25" s="11" t="n"/>
+      <c r="C25" s="11" t="n"/>
+      <c r="D25" s="11" t="n"/>
+      <c r="E25" s="11" t="n"/>
+      <c r="F25" s="11" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>